<commit_message>
Add Clarify Coach branding, QA credential tooling, and migration fixes.
Ship dual web/app brand marks, seedable QA accounts/env docs, and make pending migrations idempotent for production apply.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Clarify_AI_Enterprise_QA_Testing_Workbook.xlsx
+++ b/Clarify_AI_Enterprise_QA_Testing_Workbook.xlsx
@@ -14657,8 +14657,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
@@ -14669,7 +14669,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Test Credentials — placeholders only</t>
+          <t>Test Credentials — seeded accounts</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
@@ -14736,12 +14736,12 @@
       </c>
       <c r="B2" s="26" t="inlineStr">
         <is>
-          <t>Email (placeholder)</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C2" s="26" t="inlineStr">
         <is>
-          <t>Password (placeholder)</t>
+          <t>Password location</t>
         </is>
       </c>
       <c r="D2" s="26" t="inlineStr">
@@ -14778,12 +14778,12 @@
       </c>
       <c r="B3" s="27" t="inlineStr">
         <is>
-          <t>qa.free@example.com</t>
+          <t>qa.free@clarify.ai.test</t>
         </is>
       </c>
       <c r="C3" s="27" t="inlineStr">
         <is>
-          <t>REPLACE_ME</t>
+          <t>.env.qa.local → QA_FREE_PASSWORD</t>
         </is>
       </c>
       <c r="D3" s="27" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="F3" s="27" t="inlineStr">
         <is>
-          <t>Replace after seeding — never commit real prod secrets</t>
+          <t>Seeded by npm run qa:seed-accounts — never commit passwords</t>
         </is>
       </c>
       <c r="G3" s="27" t="inlineStr">
@@ -14816,12 +14816,12 @@
       </c>
       <c r="B4" s="28" t="inlineStr">
         <is>
-          <t>qa.pro@example.com</t>
+          <t>qa.pro@clarify.ai.test</t>
         </is>
       </c>
       <c r="C4" s="28" t="inlineStr">
         <is>
-          <t>REPLACE_ME</t>
+          <t>.env.qa.local → QA_PRO_PASSWORD</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
@@ -14849,32 +14849,32 @@
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Max / Elite</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>qa.max@example.com</t>
+          <t>qa.max@clarify.ai.test</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>REPLACE_ME</t>
+          <t>.env.qa.local → QA_MAX_PASSWORD</t>
         </is>
       </c>
       <c r="D5" s="27" t="inlineStr">
         <is>
-          <t>elite</t>
+          <t>enterprise</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="F5" s="27" t="inlineStr">
         <is>
-          <t>Priority models gate</t>
+          <t>Workbook Max/Elite maps to plan_id=enterprise</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
@@ -14892,17 +14892,17 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>qa.admin@example.com</t>
+          <t>qa.admin@clarify.ai.test</t>
         </is>
       </c>
       <c r="C6" s="28" t="inlineStr">
         <is>
-          <t>REPLACE_ME</t>
+          <t>.env.qa.local → QA_ADMIN_PASSWORD</t>
         </is>
       </c>
       <c r="D6" s="28" t="inlineStr">
         <is>
-          <t>pro+</t>
+          <t>enterprise</t>
         </is>
       </c>
       <c r="E6" s="28" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>profiles.role = admin</t>
+          <t>user_roles.admin via seed script</t>
         </is>
       </c>
       <c r="G6" s="28" t="inlineStr">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="F8" s="28" t="inlineStr">
         <is>
-          <t>INR one-time Order — no auto-renew (BUG-OPEN-01)</t>
+          <t>INR one-time Order — no auto-renew (BUG-OPEN-01); keys not in .env.local yet</t>
         </is>
       </c>
       <c r="G8" s="28" t="inlineStr">
@@ -15029,8 +15029,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
@@ -15143,7 +15143,7 @@
       </c>
       <c r="C3" s="27" t="inlineStr">
         <is>
-          <t>local / linked</t>
+          <t>qzgvjrvtkwlzxpmlddkx (linked)</t>
         </is>
       </c>
       <c r="D3" s="27" t="inlineStr">
@@ -15165,17 +15165,17 @@
     <row r="4">
       <c r="A4" s="28" t="inlineStr">
         <is>
-          <t>Staging</t>
+          <t>Staging / closed beta</t>
         </is>
       </c>
       <c r="B4" s="28" t="inlineStr">
         <is>
-          <t>https://STAGING_HOST_REPLACE</t>
+          <t>https://clarify.ai.sltfinanceindia.com</t>
         </is>
       </c>
       <c r="C4" s="28" t="inlineStr">
         <is>
-          <t>staging project ref</t>
+          <t>qzgvjrvtkwlzxpmlddkx</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
@@ -15190,7 +15190,7 @@
       </c>
       <c r="F4" s="28" t="inlineStr">
         <is>
-          <t>Primary QA target — set BaseURL cell B3 used by Feature Deep Links</t>
+          <t>Primary QA target — same project as prod until separate staging exists</t>
         </is>
       </c>
     </row>
@@ -15202,12 +15202,12 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>https://PROD_HOST_REPLACE</t>
+          <t>https://clarify.ai.sltfinanceindia.com</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>prod project ref</t>
+          <t>qzgvjrvtkwlzxpmlddkx</t>
         </is>
       </c>
       <c r="D5" s="27" t="inlineStr">
@@ -15222,7 +15222,7 @@
       </c>
       <c r="F5" s="27" t="inlineStr">
         <is>
-          <t>No destructive admin tests</t>
+          <t>Prefer seeded QA_* users; avoid destructive admin tests on shared data</t>
         </is>
       </c>
     </row>

</xml_diff>